<commit_message>
Unificar la cuenta de días a la fecha del evento
Del 3 de septiembre al 15 de octubre de 2026 hay 42 días, no 41. La hoja
"Plan 7 días" calcula esa diferencia con una fórmula, así que el texto
quedaba contradiciendo a la celda de al lado. Corregido en el dossier
markdown y en el workbook.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GYpukWA3k5ZCfL16Xb3qT1
</commit_message>
<xml_diff>
--- a/docs/propuestas/Circulo-MAV-Medellin-Directorio-de-locaciones.xlsx
+++ b/docs/propuestas/Circulo-MAV-Medellin-Directorio-de-locaciones.xlsx
@@ -2369,7 +2369,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Con 41 días a la fecha del evento, la disponibilidad manda sobre la preferencia: no se elige la locación, se elige entre las que digan sí.</t>
+          <t>Con 42 días a la fecha del evento, la disponibilidad manda sobre la preferencia: no se elige la locación, se elige entre las que digan sí.</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Anticipo, contrato con cláusula de lluvia y bloqueo de catering, sonido, iluminación y equipo de foto y video. En 41 días los proveedores son el segundo cuello de botella.</t>
+          <t>Anticipo, contrato con cláusula de lluvia y bloqueo de catering, sonido, iluminación y equipo de foto y video. En 42 días los proveedores son el segundo cuello de botella.</t>
         </is>
       </c>
       <c r="E12" s="9" t="n"/>

</xml_diff>

<commit_message>
Agregar propuesta a cliente y las tres locaciones cotizadas
Propuesta Círculo Íntimo para Valentina Ortiz: concepto, guion de las
cuatro horas anclado en la hora dorada, los tres escenarios cotizados con
inclusiones y precio, comparación de inversión y recomendación.

Las tres locaciones se suman al directorio con sus contactos, capacidades
y tarifas:
- Fábula: $5.000.000 COP, que es la tarifa de lunes a jueves y el 15/10
  es jueves. El sábado cuesta $16.800.000.
- Montpellier: $3.000.000 COP, con inclusiones por confirmar.
- Centro de Eventos El Tesoro: tarifa pendiente; el Hall 1 recibe 120 en
  auditorio.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GYpukWA3k5ZCfL16Xb3qT1
</commit_message>
<xml_diff>
--- a/docs/propuestas/Circulo-MAV-Medellin-Directorio-de-locaciones.xlsx
+++ b/docs/propuestas/Circulo-MAV-Medellin-Directorio-de-locaciones.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Plan 7 días" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Locaciones'!$A$5:$V$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Locaciones'!$A$5:$V$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -601,7 +601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V16"/>
+  <dimension ref="A1:V19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1816,8 +1816,306 @@
         </is>
       </c>
     </row>
+    <row r="17" ht="88" customHeight="1">
+      <c r="A17" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Fábula (4ST Group)</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>COTIZADA — casa de bodas y eventos</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Zona campestre de Medellín</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Ver ubicación en 4stgroup.com (Google Maps / Waze)</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="n"/>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>200 invitadas. Salón principal cerrado + zona de ceremonia al aire libre + zonas verdes. 2 salas VIP para la anfitriona. Cocina de ensamble. Parqueadero ~100 vehículos</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Sí, holgadas</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>Salón cubierto; exterior requiere carpa (no incluida)</t>
+        </is>
+      </c>
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>WhatsApp +57 305 261 8122</t>
+        </is>
+      </c>
+      <c r="K17" s="7" t="inlineStr">
+        <is>
+          <t>+57 305 261 8122</t>
+        </is>
+      </c>
+      <c r="L17" s="7" t="inlineStr">
+        <is>
+          <t>Formulario en 4stgroup.com</t>
+        </is>
+      </c>
+      <c r="M17" s="7" t="inlineStr">
+        <is>
+          <t>4stgroup.com/fabula-salon-de-bodas-eventos</t>
+        </is>
+      </c>
+      <c r="N17" s="7" t="inlineStr">
+        <is>
+          <t>Externo (cocina de ensamble en sitio)</t>
+        </is>
+      </c>
+      <c r="O17" s="7" t="inlineStr">
+        <is>
+          <t>COTIZADO $5.000.000 COP (tarifa lun-jue; el 15/10 es jueves) = $41.667 por invitada. Vie $12.200.000 · Sáb $16.800.000 · Dom/festivo $8.400.000 · Hora extra $800.000 · Calentador $150.000 c/u. Evento de 8 horas; cierre dom-jue hasta medianoche</t>
+        </is>
+      </c>
+      <c r="P17" s="7" t="inlineStr">
+        <is>
+          <t>Incluye 200 sillas Cross negras, 20 mesas rectangulares de madera (6 lugares x 20 = 120 exactos), iluminación de salón y jardines, planta eléctrica de respaldo y 2 salas VIP. 8 h de contrato = 4 h de montaje sobre una velada de 4 h</t>
+        </is>
+      </c>
+      <c r="Q17" s="7" t="inlineStr">
+        <is>
+          <t>No incluye catering, sonido, decoración ni carpas. Falta confirmar el tiempo de traslado real desde El Poblado</t>
+        </is>
+      </c>
+      <c r="R17" s="9" t="inlineStr">
+        <is>
+          <t>Cotizada</t>
+        </is>
+      </c>
+      <c r="S17" s="10" t="n"/>
+      <c r="T17" s="9" t="n"/>
+      <c r="U17" s="9" t="inlineStr">
+        <is>
+          <t>Pedir hold 48 h + cotización de carpa transparente</t>
+        </is>
+      </c>
+      <c r="V17" s="7" t="inlineStr">
+        <is>
+          <t>4stgroup.com/fabula-salon-de-bodas-eventos</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="88" customHeight="1">
+      <c r="A18" s="11" t="n">
+        <v>13</v>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>Montpellier Casa Campestre</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>COTIZADA — casa campestre</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Loma del Escobero, Envigado (finca Lorena)</t>
+        </is>
+      </c>
+      <c r="E18" s="13" t="inlineStr">
+        <is>
+          <t>Loma del Escobero, a 10 min del parque de Envigado</t>
+        </is>
+      </c>
+      <c r="F18" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="G18" s="13" t="inlineStr">
+        <is>
+          <t>Salón Barceló 150 · Zona verde 150. Jardines, kiosco, zona BBQ, baños y parqueaderos propios</t>
+        </is>
+      </c>
+      <c r="H18" s="13" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I18" s="13" t="inlineStr">
+        <is>
+          <t>Salón cubierto; zona verde descubierta</t>
+        </is>
+      </c>
+      <c r="J18" s="13" t="inlineStr">
+        <is>
+          <t>+57 311 313 1780</t>
+        </is>
+      </c>
+      <c r="K18" s="13" t="inlineStr">
+        <is>
+          <t>+57 311 313 1780</t>
+        </is>
+      </c>
+      <c r="L18" s="13" t="inlineStr">
+        <is>
+          <t>montpelliercasacampestre@gmail.com</t>
+        </is>
+      </c>
+      <c r="M18" s="13" t="inlineStr">
+        <is>
+          <t>montpelliercasacampestre.com</t>
+        </is>
+      </c>
+      <c r="N18" s="13" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
+      <c r="O18" s="13" t="inlineStr">
+        <is>
+          <t>COTIZADO $3.000.000 COP = $25.000 por invitada. $2.000.000 menos que Fábula</t>
+        </is>
+      </c>
+      <c r="P18" s="13" t="inlineStr">
+        <is>
+          <t>La más accesible y la más cercana a la ciudad. Vista abierta sobre Medellín: es lo primero que comentan quienes la visitan. Combinación salón cubierto + jardín, que es justo lo que pide el guion</t>
+        </is>
+      </c>
+      <c r="Q18" s="13" t="inlineStr">
+        <is>
+          <t>Falta por escrito: qué mobiliario incluye la tarifa, cuántas horas cubre, desde qué hora se monta, si el catering es propio o externo y el plan de lluvia</t>
+        </is>
+      </c>
+      <c r="R18" s="9" t="inlineStr">
+        <is>
+          <t>Cotizada</t>
+        </is>
+      </c>
+      <c r="S18" s="10" t="n"/>
+      <c r="T18" s="9" t="n"/>
+      <c r="U18" s="9" t="inlineStr">
+        <is>
+          <t>Pedir por escrito inclusiones, horas de montaje y plan de lluvia</t>
+        </is>
+      </c>
+      <c r="V18" s="13" t="inlineStr">
+        <is>
+          <t>montpelliercasacampestre.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="88" customHeight="1">
+      <c r="A19" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Centro de Eventos El Tesoro (CET)</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>COTIZADA — centro de convenciones</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Parque Comercial El Tesoro, El Poblado</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>Parque Comercial El Tesoro, El Poblado</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>Hall 1: 120 auditorio. Hall 2: 70 banquete. Salón 1: 400 aud. · Salón 2: 340 aud. · Salón 3: 500 aud. · Salones 2+3: 750 aud. (1.100 m²). Centro María Lucía Cossio: 1.200 pax / 2.000 m²</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Sí (Hall 1, formato auditorio)</t>
+        </is>
+      </c>
+      <c r="I19" s="7" t="inlineStr">
+        <is>
+          <t>Sí, totalmente cubierto y climatizado</t>
+        </is>
+      </c>
+      <c r="J19" s="7" t="inlineStr">
+        <is>
+          <t>+57 604 321 1010</t>
+        </is>
+      </c>
+      <c r="K19" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L19" s="7" t="inlineStr">
+        <is>
+          <t>Vía eltesoro.com.co</t>
+        </is>
+      </c>
+      <c r="M19" s="7" t="inlineStr">
+        <is>
+          <t>eltesoro.com.co/cet-centro-de-eventos-el-tesoro</t>
+        </is>
+      </c>
+      <c r="N19" s="7" t="inlineStr">
+        <is>
+          <t>Catering disponible / proveedores del centro</t>
+        </is>
+      </c>
+      <c r="O19" s="7" t="inlineStr">
+        <is>
+          <t>TARIFA PENDIENTE. Al pedirla, aclarar franja de tarde 15:00-21:00 y preguntar por el Hall 1, no por los salones grandes</t>
+        </is>
+      </c>
+      <c r="P19" s="7" t="inlineStr">
+        <is>
+          <t>Riesgo de lluvia nulo. Paneles acústicos divisorios, proyectores de 7.000-8.000 lúmenes, wifi de alta calidad y 13 puntos de acceso. Parqueadero y accesos del centro comercial; hoteles y restaurantes a pie</t>
+        </is>
+      </c>
+      <c r="Q19" s="7" t="inlineStr">
+        <is>
+          <t>Estética corporativa, no de velada. Sin exterior propio: no hay hora dorada. Contexto de centro comercial: cuesta sostener la sensación de círculo cerrado</t>
+        </is>
+      </c>
+      <c r="R19" s="9" t="inlineStr">
+        <is>
+          <t>Contactado</t>
+        </is>
+      </c>
+      <c r="S19" s="10" t="n"/>
+      <c r="T19" s="9" t="n"/>
+      <c r="U19" s="9" t="inlineStr">
+        <is>
+          <t>Solicitar tarifa del Hall 1 para franja de tarde</t>
+        </is>
+      </c>
+      <c r="V19" s="7" t="inlineStr">
+        <is>
+          <t>eltesoro.com.co/cet-centro-de-eventos-el-tesoro/salones-y-espacios</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:V16"/>
+  <autoFilter ref="A5:V19"/>
   <mergeCells count="3">
     <mergeCell ref="A2:V2"/>
     <mergeCell ref="A1:V1"/>

</xml_diff>

<commit_message>
Agregar el presupuesto integral de la velada
Presupuesto de producción completa para 120 invitadas en Fábula: locación
y carpa, gastronomía, producción técnica, ambientación, contenido,
experiencia y operación, más 12% de dirección y 8% de imprevistos.
Total $49.032.000 a $90.048.000 COP, o sea $408.600 a $750.400 por
invitada.

Va como rango porque solo las líneas de Fábula son precios de proveedor;
el resto son rangos de mercado de Medellín tomados de referencias
publicadas para eventos de 120 a 200 personas, marcados como tales en la
hoja para que se reemplacen por cotizaciones firmes.

La hoja "Presupuesto" del workbook calcula todo con fórmulas a partir de
tres variables editables: número de invitadas, porcentaje de honorarios y
porcentaje de imprevistos.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GYpukWA3k5ZCfL16Xb3qT1
</commit_message>
<xml_diff>
--- a/docs/propuestas/Circulo-MAV-Medellin-Directorio-de-locaciones.xlsx
+++ b/docs/propuestas/Circulo-MAV-Medellin-Directorio-de-locaciones.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="Locaciones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Matriz de decisión" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Checklist de llamada" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Plan 7 días" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Presupuesto" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Matriz de decisión" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Checklist de llamada" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Plan 7 días" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Locaciones'!$A$5:$V$19</definedName>
@@ -21,10 +22,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -106,8 +109,30 @@
       <color rgb="FF0000FF"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF0000FF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF006400"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF6B5F66"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF8A6E22"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -127,6 +152,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF7F4F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEDE7E9"/>
       </patternFill>
     </fill>
   </fills>
@@ -156,7 +186,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -235,6 +265,106 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="14" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2136,6 +2266,1241 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="29" t="inlineStr">
+        <is>
+          <t>PRESUPUESTO INTEGRAL — Círculo Íntimo MAV · Fábula</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>120 invitadas · jueves 15 de octubre de 2026 · 16:00 a 20:00 · valores en pesos colombianos</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="17" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Celdas en azul = variables editables (invitadas, honorarios, imprevistos y precios unitarios). Todo lo demás son fórmulas: cambiá una variable y el total se recalcula.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="30" t="inlineStr">
+        <is>
+          <t>Invitadas</t>
+        </is>
+      </c>
+      <c r="B5" s="31" t="n">
+        <v>120</v>
+      </c>
+      <c r="C5" s="30" t="inlineStr">
+        <is>
+          <t>Honorarios Aura</t>
+        </is>
+      </c>
+      <c r="D5" s="32" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E5" s="30" t="inlineStr">
+        <is>
+          <t>Imprevistos</t>
+        </is>
+      </c>
+      <c r="F5" s="32" t="n">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="33" t="inlineStr">
+        <is>
+          <t>Rubro</t>
+        </is>
+      </c>
+      <c r="B7" s="33" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="C7" s="33" t="inlineStr">
+        <is>
+          <t>Cant.</t>
+        </is>
+      </c>
+      <c r="D7" s="33" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="E7" s="33" t="inlineStr">
+        <is>
+          <t>Unitario desde</t>
+        </is>
+      </c>
+      <c r="F7" s="33" t="inlineStr">
+        <is>
+          <t>Unitario hasta</t>
+        </is>
+      </c>
+      <c r="G7" s="33" t="inlineStr">
+        <is>
+          <t>Subtotal desde</t>
+        </is>
+      </c>
+      <c r="H7" s="33" t="inlineStr">
+        <is>
+          <t>Subtotal hasta</t>
+        </is>
+      </c>
+      <c r="I7" s="33" t="inlineStr">
+        <is>
+          <t>% del total</t>
+        </is>
+      </c>
+      <c r="J7" s="33" t="inlineStr">
+        <is>
+          <t>Estado del precio</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="34" t="inlineStr">
+        <is>
+          <t>Locación</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>Alquiler Fábula · jueves, 8 horas</t>
+        </is>
+      </c>
+      <c r="C8" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="36" t="inlineStr">
+        <is>
+          <t>evento</t>
+        </is>
+      </c>
+      <c r="E8" s="37" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="F8" s="37" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="G8" s="38">
+        <f>C8*E8</f>
+        <v/>
+      </c>
+      <c r="H8" s="38">
+        <f>C8*F8</f>
+        <v/>
+      </c>
+      <c r="I8" s="39">
+        <f>H8/H$30</f>
+        <v/>
+      </c>
+      <c r="J8" s="40" t="inlineStr">
+        <is>
+          <t>CONFIRMADO — tarifa lun a jue publicada</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="41" t="inlineStr">
+        <is>
+          <t>Locación</t>
+        </is>
+      </c>
+      <c r="B9" s="42" t="inlineStr">
+        <is>
+          <t>Carpa transparente para el jardín (~180 m²)</t>
+        </is>
+      </c>
+      <c r="C9" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="44" t="inlineStr">
+        <is>
+          <t>montaje</t>
+        </is>
+      </c>
+      <c r="E9" s="45" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="F9" s="45" t="n">
+        <v>4500000</v>
+      </c>
+      <c r="G9" s="46">
+        <f>C9*E9</f>
+        <v/>
+      </c>
+      <c r="H9" s="46">
+        <f>C9*F9</f>
+        <v/>
+      </c>
+      <c r="I9" s="47">
+        <f>H9/H$30</f>
+        <v/>
+      </c>
+      <c r="J9" s="48" t="inlineStr">
+        <is>
+          <t>Estimado de mercado</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="34" t="inlineStr">
+        <is>
+          <t>Locación</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>Calentadores exteriores</t>
+        </is>
+      </c>
+      <c r="C10" s="35" t="n">
+        <v>6</v>
+      </c>
+      <c r="D10" s="36" t="inlineStr">
+        <is>
+          <t>unidad</t>
+        </is>
+      </c>
+      <c r="E10" s="37" t="n">
+        <v>150000</v>
+      </c>
+      <c r="F10" s="37" t="n">
+        <v>150000</v>
+      </c>
+      <c r="G10" s="38">
+        <f>C10*E10</f>
+        <v/>
+      </c>
+      <c r="H10" s="38">
+        <f>C10*F10</f>
+        <v/>
+      </c>
+      <c r="I10" s="39">
+        <f>H10/H$30</f>
+        <v/>
+      </c>
+      <c r="J10" s="40" t="inlineStr">
+        <is>
+          <t>CONFIRMADO — precio unitario de Fábula</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="41" t="inlineStr">
+        <is>
+          <t>Locación</t>
+        </is>
+      </c>
+      <c r="B11" s="42" t="inlineStr">
+        <is>
+          <t>Hora adicional (reserva por si se extiende)</t>
+        </is>
+      </c>
+      <c r="C11" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="44" t="inlineStr">
+        <is>
+          <t>hora</t>
+        </is>
+      </c>
+      <c r="E11" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="45" t="n">
+        <v>800000</v>
+      </c>
+      <c r="G11" s="46">
+        <f>C11*E11</f>
+        <v/>
+      </c>
+      <c r="H11" s="46">
+        <f>C11*F11</f>
+        <v/>
+      </c>
+      <c r="I11" s="47">
+        <f>H11/H$30</f>
+        <v/>
+      </c>
+      <c r="J11" s="49" t="inlineStr">
+        <is>
+          <t>CONFIRMADO — precio unitario de Fábula</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="34" t="inlineStr">
+        <is>
+          <t>Gastronomía</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>Catering: recepción, estaciones y postre</t>
+        </is>
+      </c>
+      <c r="C12" s="35">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="D12" s="36" t="inlineStr">
+        <is>
+          <t>invitada</t>
+        </is>
+      </c>
+      <c r="E12" s="37" t="n">
+        <v>45000</v>
+      </c>
+      <c r="F12" s="37" t="n">
+        <v>70000</v>
+      </c>
+      <c r="G12" s="38">
+        <f>C12*E12</f>
+        <v/>
+      </c>
+      <c r="H12" s="38">
+        <f>C12*F12</f>
+        <v/>
+      </c>
+      <c r="I12" s="39">
+        <f>H12/H$30</f>
+        <v/>
+      </c>
+      <c r="J12" s="50" t="inlineStr">
+        <is>
+          <t>Estimado — mercado Medellín $15.000 a $50.000; vamos por encima del tope</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="41" t="inlineStr">
+        <is>
+          <t>Gastronomía</t>
+        </is>
+      </c>
+      <c r="B13" s="42" t="inlineStr">
+        <is>
+          <t>Barra y coctelería de autor</t>
+        </is>
+      </c>
+      <c r="C13" s="43">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="D13" s="44" t="inlineStr">
+        <is>
+          <t>invitada</t>
+        </is>
+      </c>
+      <c r="E13" s="45" t="n">
+        <v>18000</v>
+      </c>
+      <c r="F13" s="45" t="n">
+        <v>32000</v>
+      </c>
+      <c r="G13" s="46">
+        <f>C13*E13</f>
+        <v/>
+      </c>
+      <c r="H13" s="46">
+        <f>C13*F13</f>
+        <v/>
+      </c>
+      <c r="I13" s="47">
+        <f>H13/H$30</f>
+        <v/>
+      </c>
+      <c r="J13" s="48" t="inlineStr">
+        <is>
+          <t>Estimado de mercado</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="34" t="inlineStr">
+        <is>
+          <t>Gastronomía</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>Staff de servicio y bar</t>
+        </is>
+      </c>
+      <c r="C14" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="D14" s="36" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="E14" s="37" t="n">
+        <v>180000</v>
+      </c>
+      <c r="F14" s="37" t="n">
+        <v>280000</v>
+      </c>
+      <c r="G14" s="38">
+        <f>C14*E14</f>
+        <v/>
+      </c>
+      <c r="H14" s="38">
+        <f>C14*F14</f>
+        <v/>
+      </c>
+      <c r="I14" s="39">
+        <f>H14/H$30</f>
+        <v/>
+      </c>
+      <c r="J14" s="50" t="inlineStr">
+        <is>
+          <t>Estimado — una persona cada 12 invitadas</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="41" t="inlineStr">
+        <is>
+          <t>Producción técnica</t>
+        </is>
+      </c>
+      <c r="B15" s="42" t="inlineStr">
+        <is>
+          <t>Sonido y microfonía inalámbrica</t>
+        </is>
+      </c>
+      <c r="C15" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="44" t="inlineStr">
+        <is>
+          <t>servicio</t>
+        </is>
+      </c>
+      <c r="E15" s="45" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="F15" s="45" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="G15" s="46">
+        <f>C15*E15</f>
+        <v/>
+      </c>
+      <c r="H15" s="46">
+        <f>C15*F15</f>
+        <v/>
+      </c>
+      <c r="I15" s="47">
+        <f>H15/H$30</f>
+        <v/>
+      </c>
+      <c r="J15" s="48" t="inlineStr">
+        <is>
+          <t>Estimado de mercado</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="34" t="inlineStr">
+        <is>
+          <t>Producción técnica</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>Iluminación escénica y de jardín</t>
+        </is>
+      </c>
+      <c r="C16" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="36" t="inlineStr">
+        <is>
+          <t>servicio</t>
+        </is>
+      </c>
+      <c r="E16" s="37" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="F16" s="37" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="G16" s="38">
+        <f>C16*E16</f>
+        <v/>
+      </c>
+      <c r="H16" s="38">
+        <f>C16*F16</f>
+        <v/>
+      </c>
+      <c r="I16" s="39">
+        <f>H16/H$30</f>
+        <v/>
+      </c>
+      <c r="J16" s="50" t="inlineStr">
+        <is>
+          <t>Estimado de mercado</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="41" t="inlineStr">
+        <is>
+          <t>Producción técnica</t>
+        </is>
+      </c>
+      <c r="B17" s="42" t="inlineStr">
+        <is>
+          <t>Pantalla LED o proyección con operador</t>
+        </is>
+      </c>
+      <c r="C17" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="44" t="inlineStr">
+        <is>
+          <t>servicio</t>
+        </is>
+      </c>
+      <c r="E17" s="45" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="F17" s="45" t="n">
+        <v>3500000</v>
+      </c>
+      <c r="G17" s="46">
+        <f>C17*E17</f>
+        <v/>
+      </c>
+      <c r="H17" s="46">
+        <f>C17*F17</f>
+        <v/>
+      </c>
+      <c r="I17" s="47">
+        <f>H17/H$30</f>
+        <v/>
+      </c>
+      <c r="J17" s="48" t="inlineStr">
+        <is>
+          <t>Estimado de mercado</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="34" t="inlineStr">
+        <is>
+          <t>Producción técnica</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>Tarima y backdrop</t>
+        </is>
+      </c>
+      <c r="C18" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="36" t="inlineStr">
+        <is>
+          <t>montaje</t>
+        </is>
+      </c>
+      <c r="E18" s="37" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="F18" s="37" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="G18" s="38">
+        <f>C18*E18</f>
+        <v/>
+      </c>
+      <c r="H18" s="38">
+        <f>C18*F18</f>
+        <v/>
+      </c>
+      <c r="I18" s="39">
+        <f>H18/H$30</f>
+        <v/>
+      </c>
+      <c r="J18" s="50" t="inlineStr">
+        <is>
+          <t>Estimado de mercado</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="41" t="inlineStr">
+        <is>
+          <t>Ambientación</t>
+        </is>
+      </c>
+      <c r="B19" s="42" t="inlineStr">
+        <is>
+          <t>Diseño floral y ambientación</t>
+        </is>
+      </c>
+      <c r="C19" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="44" t="inlineStr">
+        <is>
+          <t>servicio</t>
+        </is>
+      </c>
+      <c r="E19" s="45" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="F19" s="45" t="n">
+        <v>7000000</v>
+      </c>
+      <c r="G19" s="46">
+        <f>C19*E19</f>
+        <v/>
+      </c>
+      <c r="H19" s="46">
+        <f>C19*F19</f>
+        <v/>
+      </c>
+      <c r="I19" s="47">
+        <f>H19/H$30</f>
+        <v/>
+      </c>
+      <c r="J19" s="48" t="inlineStr">
+        <is>
+          <t>Estimado — mercado Medellín $3M a $10M</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="34" t="inlineStr">
+        <is>
+          <t>Ambientación</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="inlineStr">
+        <is>
+          <t>Mobiliario lounge, barras y mantelería</t>
+        </is>
+      </c>
+      <c r="C20" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="36" t="inlineStr">
+        <is>
+          <t>servicio</t>
+        </is>
+      </c>
+      <c r="E20" s="37" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="F20" s="37" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="G20" s="38">
+        <f>C20*E20</f>
+        <v/>
+      </c>
+      <c r="H20" s="38">
+        <f>C20*F20</f>
+        <v/>
+      </c>
+      <c r="I20" s="39">
+        <f>H20/H$30</f>
+        <v/>
+      </c>
+      <c r="J20" s="50" t="inlineStr">
+        <is>
+          <t>Estimado — bajo porque Fábula ya incluye sillas y mesas</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="41" t="inlineStr">
+        <is>
+          <t>Contenido</t>
+        </is>
+      </c>
+      <c r="B21" s="42" t="inlineStr">
+        <is>
+          <t>Fotografía · dos fotógrafas</t>
+        </is>
+      </c>
+      <c r="C21" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="44" t="inlineStr">
+        <is>
+          <t>servicio</t>
+        </is>
+      </c>
+      <c r="E21" s="45" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="F21" s="45" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="G21" s="46">
+        <f>C21*E21</f>
+        <v/>
+      </c>
+      <c r="H21" s="46">
+        <f>C21*F21</f>
+        <v/>
+      </c>
+      <c r="I21" s="47">
+        <f>H21/H$30</f>
+        <v/>
+      </c>
+      <c r="J21" s="48" t="inlineStr">
+        <is>
+          <t>Estimado — mercado Medellín $2M a $5M</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="34" t="inlineStr">
+        <is>
+          <t>Contenido</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>Video · equipo de dos y edición</t>
+        </is>
+      </c>
+      <c r="C22" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="36" t="inlineStr">
+        <is>
+          <t>servicio</t>
+        </is>
+      </c>
+      <c r="E22" s="37" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="F22" s="37" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="G22" s="38">
+        <f>C22*E22</f>
+        <v/>
+      </c>
+      <c r="H22" s="38">
+        <f>C22*F22</f>
+        <v/>
+      </c>
+      <c r="I22" s="39">
+        <f>H22/H$30</f>
+        <v/>
+      </c>
+      <c r="J22" s="50" t="inlineStr">
+        <is>
+          <t>Estimado — mercado Medellín $3M a $7M</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="41" t="inlineStr">
+        <is>
+          <t>Experiencia</t>
+        </is>
+      </c>
+      <c r="B23" s="42" t="inlineStr">
+        <is>
+          <t>Música en vivo</t>
+        </is>
+      </c>
+      <c r="C23" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="44" t="inlineStr">
+        <is>
+          <t>servicio</t>
+        </is>
+      </c>
+      <c r="E23" s="45" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="F23" s="45" t="n">
+        <v>3500000</v>
+      </c>
+      <c r="G23" s="46">
+        <f>C23*E23</f>
+        <v/>
+      </c>
+      <c r="H23" s="46">
+        <f>C23*F23</f>
+        <v/>
+      </c>
+      <c r="I23" s="47">
+        <f>H23/H$30</f>
+        <v/>
+      </c>
+      <c r="J23" s="48" t="inlineStr">
+        <is>
+          <t>Estimado — mercado Medellín $3M a $8M con show completo</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="34" t="inlineStr">
+        <is>
+          <t>Experiencia</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="inlineStr">
+        <is>
+          <t>Detalle para cada invitada</t>
+        </is>
+      </c>
+      <c r="C24" s="35">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="D24" s="36" t="inlineStr">
+        <is>
+          <t>invitada</t>
+        </is>
+      </c>
+      <c r="E24" s="37" t="n">
+        <v>35000</v>
+      </c>
+      <c r="F24" s="37" t="n">
+        <v>80000</v>
+      </c>
+      <c r="G24" s="38">
+        <f>C24*E24</f>
+        <v/>
+      </c>
+      <c r="H24" s="38">
+        <f>C24*F24</f>
+        <v/>
+      </c>
+      <c r="I24" s="39">
+        <f>H24/H$30</f>
+        <v/>
+      </c>
+      <c r="J24" s="50" t="inlineStr">
+        <is>
+          <t>Estimado — define mucho el total</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="28" customHeight="1">
+      <c r="A25" s="41" t="inlineStr">
+        <is>
+          <t>Experiencia</t>
+        </is>
+      </c>
+      <c r="B25" s="42" t="inlineStr">
+        <is>
+          <t>Papelería, señalética y nombres a mano</t>
+        </is>
+      </c>
+      <c r="C25" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="44" t="inlineStr">
+        <is>
+          <t>servicio</t>
+        </is>
+      </c>
+      <c r="E25" s="45" t="n">
+        <v>600000</v>
+      </c>
+      <c r="F25" s="45" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="G25" s="46">
+        <f>C25*E25</f>
+        <v/>
+      </c>
+      <c r="H25" s="46">
+        <f>C25*F25</f>
+        <v/>
+      </c>
+      <c r="I25" s="47">
+        <f>H25/H$30</f>
+        <v/>
+      </c>
+      <c r="J25" s="48" t="inlineStr">
+        <is>
+          <t>Estimado de mercado</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="34" t="inlineStr">
+        <is>
+          <t>Operación</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="inlineStr">
+        <is>
+          <t>Transporte y logística de montaje</t>
+        </is>
+      </c>
+      <c r="C26" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="36" t="inlineStr">
+        <is>
+          <t>servicio</t>
+        </is>
+      </c>
+      <c r="E26" s="37" t="n">
+        <v>800000</v>
+      </c>
+      <c r="F26" s="37" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="G26" s="38">
+        <f>C26*E26</f>
+        <v/>
+      </c>
+      <c r="H26" s="38">
+        <f>C26*F26</f>
+        <v/>
+      </c>
+      <c r="I26" s="39">
+        <f>H26/H$30</f>
+        <v/>
+      </c>
+      <c r="J26" s="50" t="inlineStr">
+        <is>
+          <t>Estimado de mercado</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="51" t="inlineStr">
+        <is>
+          <t>SUBTOTAL DIRECTO</t>
+        </is>
+      </c>
+      <c r="B27" s="51" t="n"/>
+      <c r="C27" s="51" t="n"/>
+      <c r="D27" s="51" t="n"/>
+      <c r="E27" s="51" t="n"/>
+      <c r="F27" s="51" t="n"/>
+      <c r="G27" s="52">
+        <f>SUM(G8:G26)</f>
+        <v/>
+      </c>
+      <c r="H27" s="52">
+        <f>SUM(H8:H26)</f>
+        <v/>
+      </c>
+      <c r="I27" s="51" t="n"/>
+      <c r="J27" s="51" t="n"/>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="53" t="inlineStr">
+        <is>
+          <t>Producción y dirección · Aura Productions</t>
+        </is>
+      </c>
+      <c r="B28" s="53" t="n"/>
+      <c r="C28" s="53" t="n"/>
+      <c r="D28" s="53" t="n"/>
+      <c r="E28" s="53" t="n"/>
+      <c r="F28" s="53" t="n"/>
+      <c r="G28" s="54">
+        <f>G27*$D$5</f>
+        <v/>
+      </c>
+      <c r="H28" s="54">
+        <f>H27*$D$5</f>
+        <v/>
+      </c>
+      <c r="I28" s="53" t="n"/>
+      <c r="J28" s="53" t="n"/>
+    </row>
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" s="53" t="inlineStr">
+        <is>
+          <t>Imprevistos</t>
+        </is>
+      </c>
+      <c r="B29" s="53" t="n"/>
+      <c r="C29" s="53" t="n"/>
+      <c r="D29" s="53" t="n"/>
+      <c r="E29" s="53" t="n"/>
+      <c r="F29" s="53" t="n"/>
+      <c r="G29" s="54">
+        <f>G27*$F$5</f>
+        <v/>
+      </c>
+      <c r="H29" s="54">
+        <f>H27*$F$5</f>
+        <v/>
+      </c>
+      <c r="I29" s="53" t="n"/>
+      <c r="J29" s="53" t="n"/>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" s="55" t="inlineStr">
+        <is>
+          <t>TOTAL DE LA VELADA</t>
+        </is>
+      </c>
+      <c r="B30" s="55" t="n"/>
+      <c r="C30" s="55" t="n"/>
+      <c r="D30" s="55" t="n"/>
+      <c r="E30" s="55" t="n"/>
+      <c r="F30" s="55" t="n"/>
+      <c r="G30" s="56">
+        <f>G27+G28+G29</f>
+        <v/>
+      </c>
+      <c r="H30" s="56">
+        <f>H27+H28+H29</f>
+        <v/>
+      </c>
+      <c r="I30" s="55" t="n"/>
+      <c r="J30" s="55" t="n"/>
+    </row>
+    <row r="31" ht="24" customHeight="1">
+      <c r="A31" s="55" t="inlineStr">
+        <is>
+          <t>Por invitada</t>
+        </is>
+      </c>
+      <c r="B31" s="55" t="n"/>
+      <c r="C31" s="55" t="n"/>
+      <c r="D31" s="55" t="n"/>
+      <c r="E31" s="55" t="n"/>
+      <c r="F31" s="55" t="n"/>
+      <c r="G31" s="56">
+        <f>G30/$B$5</f>
+        <v/>
+      </c>
+      <c r="H31" s="56">
+        <f>H30/$B$5</f>
+        <v/>
+      </c>
+      <c r="I31" s="55" t="n"/>
+      <c r="J31" s="55" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="57" t="inlineStr">
+        <is>
+          <t>RESUMEN POR RUBRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="58" t="inlineStr">
+        <is>
+          <t>Rubro</t>
+        </is>
+      </c>
+      <c r="B34" s="58" t="inlineStr">
+        <is>
+          <t>Desde</t>
+        </is>
+      </c>
+      <c r="C34" s="58" t="inlineStr">
+        <is>
+          <t>Hasta</t>
+        </is>
+      </c>
+      <c r="D34" s="58" t="inlineStr">
+        <is>
+          <t>% del total</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="59" t="inlineStr">
+        <is>
+          <t>Locación</t>
+        </is>
+      </c>
+      <c r="B35" s="60">
+        <f>SUMIF($A$8:$A$26,$A35,$G$8:$G$26)</f>
+        <v/>
+      </c>
+      <c r="C35" s="60">
+        <f>SUMIF($A$8:$A$26,$A35,$H$8:$H$26)</f>
+        <v/>
+      </c>
+      <c r="D35" s="61">
+        <f>C35/$H$27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="59" t="inlineStr">
+        <is>
+          <t>Gastronomía</t>
+        </is>
+      </c>
+      <c r="B36" s="60">
+        <f>SUMIF($A$8:$A$26,$A36,$G$8:$G$26)</f>
+        <v/>
+      </c>
+      <c r="C36" s="60">
+        <f>SUMIF($A$8:$A$26,$A36,$H$8:$H$26)</f>
+        <v/>
+      </c>
+      <c r="D36" s="61">
+        <f>C36/$H$27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="59" t="inlineStr">
+        <is>
+          <t>Producción técnica</t>
+        </is>
+      </c>
+      <c r="B37" s="60">
+        <f>SUMIF($A$8:$A$26,$A37,$G$8:$G$26)</f>
+        <v/>
+      </c>
+      <c r="C37" s="60">
+        <f>SUMIF($A$8:$A$26,$A37,$H$8:$H$26)</f>
+        <v/>
+      </c>
+      <c r="D37" s="61">
+        <f>C37/$H$27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="59" t="inlineStr">
+        <is>
+          <t>Ambientación</t>
+        </is>
+      </c>
+      <c r="B38" s="60">
+        <f>SUMIF($A$8:$A$26,$A38,$G$8:$G$26)</f>
+        <v/>
+      </c>
+      <c r="C38" s="60">
+        <f>SUMIF($A$8:$A$26,$A38,$H$8:$H$26)</f>
+        <v/>
+      </c>
+      <c r="D38" s="61">
+        <f>C38/$H$27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="59" t="inlineStr">
+        <is>
+          <t>Contenido</t>
+        </is>
+      </c>
+      <c r="B39" s="60">
+        <f>SUMIF($A$8:$A$26,$A39,$G$8:$G$26)</f>
+        <v/>
+      </c>
+      <c r="C39" s="60">
+        <f>SUMIF($A$8:$A$26,$A39,$H$8:$H$26)</f>
+        <v/>
+      </c>
+      <c r="D39" s="61">
+        <f>C39/$H$27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="59" t="inlineStr">
+        <is>
+          <t>Experiencia</t>
+        </is>
+      </c>
+      <c r="B40" s="60">
+        <f>SUMIF($A$8:$A$26,$A40,$G$8:$G$26)</f>
+        <v/>
+      </c>
+      <c r="C40" s="60">
+        <f>SUMIF($A$8:$A$26,$A40,$H$8:$H$26)</f>
+        <v/>
+      </c>
+      <c r="D40" s="61">
+        <f>C40/$H$27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="59" t="inlineStr">
+        <is>
+          <t>Operación</t>
+        </is>
+      </c>
+      <c r="B41" s="60">
+        <f>SUMIF($A$8:$A$26,$A41,$G$8:$G$26)</f>
+        <v/>
+      </c>
+      <c r="C41" s="60">
+        <f>SUMIF($A$8:$A$26,$A41,$H$8:$H$26)</f>
+        <v/>
+      </c>
+      <c r="D41" s="61">
+        <f>C41/$H$27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" ht="52" customHeight="1">
+      <c r="A43" s="62" t="inlineStr">
+        <is>
+          <t>Cómo leer este presupuesto: solo las líneas marcadas CONFIRMADO en verde son precios reales de proveedor (Fábula). Todo lo demás son estimaciones de mercado de Medellín tomadas de rangos publicados para eventos de 120 a 200 personas, y deben reemplazarse por cotizaciones firmes antes de presentar un número cerrado. Las tres palancas que más mueven el total son el catering, el detalle para cada invitada y el diseño floral: ajustando esas tres se baja o se sube el presupuesto sin tocar la experiencia.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A43:J43"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A29:F29"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2416,7 +3781,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2640,7 +4005,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Borrar el presupuesto inventado y las 13 cards
Se elimina la hoja "Presupuesto" del workbook: salvo las tarifas de las
tres locaciones, sus cifras no tenían respaldo.

Se eliminan las 13 cards de Instagram y su archivo fuente, que
arrastraban ese mismo presupuesto y además el guion anterior, con bloques
que nunca existieron.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GYpukWA3k5ZCfL16Xb3qT1
</commit_message>
<xml_diff>
--- a/docs/propuestas/Circulo-MAV-Medellin-Directorio-de-locaciones.xlsx
+++ b/docs/propuestas/Circulo-MAV-Medellin-Directorio-de-locaciones.xlsx
@@ -8,10 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="Locaciones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Presupuesto" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Matriz de decisión" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Checklist de llamada" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Plan 7 días" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Matriz de decisión" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Checklist de llamada" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Plan 7 días" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Locaciones'!$A$5:$V$19</definedName>
@@ -160,7 +159,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -181,6 +180,50 @@
       <bottom style="thin">
         <color rgb="FFD8D0D3"/>
       </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD8D0D3"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD8D0D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD8D0D3"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD8D0D3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD8D0D3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD8D0D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD8D0D3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD8D0D3"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -2266,1241 +2309,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J43"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="46" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="29" t="inlineStr">
-        <is>
-          <t>PRESUPUESTO INTEGRAL — Círculo Íntimo MAV · Fábula</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>120 invitadas · jueves 15 de octubre de 2026 · 16:00 a 20:00 · valores en pesos colombianos</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="17" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Celdas en azul = variables editables (invitadas, honorarios, imprevistos y precios unitarios). Todo lo demás son fórmulas: cambiá una variable y el total se recalcula.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="30" t="inlineStr">
-        <is>
-          <t>Invitadas</t>
-        </is>
-      </c>
-      <c r="B5" s="31" t="n">
-        <v>120</v>
-      </c>
-      <c r="C5" s="30" t="inlineStr">
-        <is>
-          <t>Honorarios Aura</t>
-        </is>
-      </c>
-      <c r="D5" s="32" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="E5" s="30" t="inlineStr">
-        <is>
-          <t>Imprevistos</t>
-        </is>
-      </c>
-      <c r="F5" s="32" t="n">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="33" t="inlineStr">
-        <is>
-          <t>Rubro</t>
-        </is>
-      </c>
-      <c r="B7" s="33" t="inlineStr">
-        <is>
-          <t>Concepto</t>
-        </is>
-      </c>
-      <c r="C7" s="33" t="inlineStr">
-        <is>
-          <t>Cant.</t>
-        </is>
-      </c>
-      <c r="D7" s="33" t="inlineStr">
-        <is>
-          <t>Unidad</t>
-        </is>
-      </c>
-      <c r="E7" s="33" t="inlineStr">
-        <is>
-          <t>Unitario desde</t>
-        </is>
-      </c>
-      <c r="F7" s="33" t="inlineStr">
-        <is>
-          <t>Unitario hasta</t>
-        </is>
-      </c>
-      <c r="G7" s="33" t="inlineStr">
-        <is>
-          <t>Subtotal desde</t>
-        </is>
-      </c>
-      <c r="H7" s="33" t="inlineStr">
-        <is>
-          <t>Subtotal hasta</t>
-        </is>
-      </c>
-      <c r="I7" s="33" t="inlineStr">
-        <is>
-          <t>% del total</t>
-        </is>
-      </c>
-      <c r="J7" s="33" t="inlineStr">
-        <is>
-          <t>Estado del precio</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="34" t="inlineStr">
-        <is>
-          <t>Locación</t>
-        </is>
-      </c>
-      <c r="B8" s="15" t="inlineStr">
-        <is>
-          <t>Alquiler Fábula · jueves, 8 horas</t>
-        </is>
-      </c>
-      <c r="C8" s="35" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="36" t="inlineStr">
-        <is>
-          <t>evento</t>
-        </is>
-      </c>
-      <c r="E8" s="37" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="F8" s="37" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="G8" s="38">
-        <f>C8*E8</f>
-        <v/>
-      </c>
-      <c r="H8" s="38">
-        <f>C8*F8</f>
-        <v/>
-      </c>
-      <c r="I8" s="39">
-        <f>H8/H$30</f>
-        <v/>
-      </c>
-      <c r="J8" s="40" t="inlineStr">
-        <is>
-          <t>CONFIRMADO — tarifa lun a jue publicada</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="28" customHeight="1">
-      <c r="A9" s="41" t="inlineStr">
-        <is>
-          <t>Locación</t>
-        </is>
-      </c>
-      <c r="B9" s="42" t="inlineStr">
-        <is>
-          <t>Carpa transparente para el jardín (~180 m²)</t>
-        </is>
-      </c>
-      <c r="C9" s="43" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="44" t="inlineStr">
-        <is>
-          <t>montaje</t>
-        </is>
-      </c>
-      <c r="E9" s="45" t="n">
-        <v>2500000</v>
-      </c>
-      <c r="F9" s="45" t="n">
-        <v>4500000</v>
-      </c>
-      <c r="G9" s="46">
-        <f>C9*E9</f>
-        <v/>
-      </c>
-      <c r="H9" s="46">
-        <f>C9*F9</f>
-        <v/>
-      </c>
-      <c r="I9" s="47">
-        <f>H9/H$30</f>
-        <v/>
-      </c>
-      <c r="J9" s="48" t="inlineStr">
-        <is>
-          <t>Estimado de mercado</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="34" t="inlineStr">
-        <is>
-          <t>Locación</t>
-        </is>
-      </c>
-      <c r="B10" s="15" t="inlineStr">
-        <is>
-          <t>Calentadores exteriores</t>
-        </is>
-      </c>
-      <c r="C10" s="35" t="n">
-        <v>6</v>
-      </c>
-      <c r="D10" s="36" t="inlineStr">
-        <is>
-          <t>unidad</t>
-        </is>
-      </c>
-      <c r="E10" s="37" t="n">
-        <v>150000</v>
-      </c>
-      <c r="F10" s="37" t="n">
-        <v>150000</v>
-      </c>
-      <c r="G10" s="38">
-        <f>C10*E10</f>
-        <v/>
-      </c>
-      <c r="H10" s="38">
-        <f>C10*F10</f>
-        <v/>
-      </c>
-      <c r="I10" s="39">
-        <f>H10/H$30</f>
-        <v/>
-      </c>
-      <c r="J10" s="40" t="inlineStr">
-        <is>
-          <t>CONFIRMADO — precio unitario de Fábula</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="28" customHeight="1">
-      <c r="A11" s="41" t="inlineStr">
-        <is>
-          <t>Locación</t>
-        </is>
-      </c>
-      <c r="B11" s="42" t="inlineStr">
-        <is>
-          <t>Hora adicional (reserva por si se extiende)</t>
-        </is>
-      </c>
-      <c r="C11" s="43" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="44" t="inlineStr">
-        <is>
-          <t>hora</t>
-        </is>
-      </c>
-      <c r="E11" s="45" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="45" t="n">
-        <v>800000</v>
-      </c>
-      <c r="G11" s="46">
-        <f>C11*E11</f>
-        <v/>
-      </c>
-      <c r="H11" s="46">
-        <f>C11*F11</f>
-        <v/>
-      </c>
-      <c r="I11" s="47">
-        <f>H11/H$30</f>
-        <v/>
-      </c>
-      <c r="J11" s="49" t="inlineStr">
-        <is>
-          <t>CONFIRMADO — precio unitario de Fábula</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="34" t="inlineStr">
-        <is>
-          <t>Gastronomía</t>
-        </is>
-      </c>
-      <c r="B12" s="15" t="inlineStr">
-        <is>
-          <t>Catering: recepción, estaciones y postre</t>
-        </is>
-      </c>
-      <c r="C12" s="35">
-        <f>$B$5</f>
-        <v/>
-      </c>
-      <c r="D12" s="36" t="inlineStr">
-        <is>
-          <t>invitada</t>
-        </is>
-      </c>
-      <c r="E12" s="37" t="n">
-        <v>45000</v>
-      </c>
-      <c r="F12" s="37" t="n">
-        <v>70000</v>
-      </c>
-      <c r="G12" s="38">
-        <f>C12*E12</f>
-        <v/>
-      </c>
-      <c r="H12" s="38">
-        <f>C12*F12</f>
-        <v/>
-      </c>
-      <c r="I12" s="39">
-        <f>H12/H$30</f>
-        <v/>
-      </c>
-      <c r="J12" s="50" t="inlineStr">
-        <is>
-          <t>Estimado — mercado Medellín $15.000 a $50.000; vamos por encima del tope</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="41" t="inlineStr">
-        <is>
-          <t>Gastronomía</t>
-        </is>
-      </c>
-      <c r="B13" s="42" t="inlineStr">
-        <is>
-          <t>Barra y coctelería de autor</t>
-        </is>
-      </c>
-      <c r="C13" s="43">
-        <f>$B$5</f>
-        <v/>
-      </c>
-      <c r="D13" s="44" t="inlineStr">
-        <is>
-          <t>invitada</t>
-        </is>
-      </c>
-      <c r="E13" s="45" t="n">
-        <v>18000</v>
-      </c>
-      <c r="F13" s="45" t="n">
-        <v>32000</v>
-      </c>
-      <c r="G13" s="46">
-        <f>C13*E13</f>
-        <v/>
-      </c>
-      <c r="H13" s="46">
-        <f>C13*F13</f>
-        <v/>
-      </c>
-      <c r="I13" s="47">
-        <f>H13/H$30</f>
-        <v/>
-      </c>
-      <c r="J13" s="48" t="inlineStr">
-        <is>
-          <t>Estimado de mercado</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="34" t="inlineStr">
-        <is>
-          <t>Gastronomía</t>
-        </is>
-      </c>
-      <c r="B14" s="15" t="inlineStr">
-        <is>
-          <t>Staff de servicio y bar</t>
-        </is>
-      </c>
-      <c r="C14" s="35" t="n">
-        <v>10</v>
-      </c>
-      <c r="D14" s="36" t="inlineStr">
-        <is>
-          <t>persona</t>
-        </is>
-      </c>
-      <c r="E14" s="37" t="n">
-        <v>180000</v>
-      </c>
-      <c r="F14" s="37" t="n">
-        <v>280000</v>
-      </c>
-      <c r="G14" s="38">
-        <f>C14*E14</f>
-        <v/>
-      </c>
-      <c r="H14" s="38">
-        <f>C14*F14</f>
-        <v/>
-      </c>
-      <c r="I14" s="39">
-        <f>H14/H$30</f>
-        <v/>
-      </c>
-      <c r="J14" s="50" t="inlineStr">
-        <is>
-          <t>Estimado — una persona cada 12 invitadas</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="41" t="inlineStr">
-        <is>
-          <t>Producción técnica</t>
-        </is>
-      </c>
-      <c r="B15" s="42" t="inlineStr">
-        <is>
-          <t>Sonido y microfonía inalámbrica</t>
-        </is>
-      </c>
-      <c r="C15" s="43" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="44" t="inlineStr">
-        <is>
-          <t>servicio</t>
-        </is>
-      </c>
-      <c r="E15" s="45" t="n">
-        <v>1500000</v>
-      </c>
-      <c r="F15" s="45" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="G15" s="46">
-        <f>C15*E15</f>
-        <v/>
-      </c>
-      <c r="H15" s="46">
-        <f>C15*F15</f>
-        <v/>
-      </c>
-      <c r="I15" s="47">
-        <f>H15/H$30</f>
-        <v/>
-      </c>
-      <c r="J15" s="48" t="inlineStr">
-        <is>
-          <t>Estimado de mercado</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="34" t="inlineStr">
-        <is>
-          <t>Producción técnica</t>
-        </is>
-      </c>
-      <c r="B16" s="15" t="inlineStr">
-        <is>
-          <t>Iluminación escénica y de jardín</t>
-        </is>
-      </c>
-      <c r="C16" s="35" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="36" t="inlineStr">
-        <is>
-          <t>servicio</t>
-        </is>
-      </c>
-      <c r="E16" s="37" t="n">
-        <v>2000000</v>
-      </c>
-      <c r="F16" s="37" t="n">
-        <v>4000000</v>
-      </c>
-      <c r="G16" s="38">
-        <f>C16*E16</f>
-        <v/>
-      </c>
-      <c r="H16" s="38">
-        <f>C16*F16</f>
-        <v/>
-      </c>
-      <c r="I16" s="39">
-        <f>H16/H$30</f>
-        <v/>
-      </c>
-      <c r="J16" s="50" t="inlineStr">
-        <is>
-          <t>Estimado de mercado</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="41" t="inlineStr">
-        <is>
-          <t>Producción técnica</t>
-        </is>
-      </c>
-      <c r="B17" s="42" t="inlineStr">
-        <is>
-          <t>Pantalla LED o proyección con operador</t>
-        </is>
-      </c>
-      <c r="C17" s="43" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="44" t="inlineStr">
-        <is>
-          <t>servicio</t>
-        </is>
-      </c>
-      <c r="E17" s="45" t="n">
-        <v>1800000</v>
-      </c>
-      <c r="F17" s="45" t="n">
-        <v>3500000</v>
-      </c>
-      <c r="G17" s="46">
-        <f>C17*E17</f>
-        <v/>
-      </c>
-      <c r="H17" s="46">
-        <f>C17*F17</f>
-        <v/>
-      </c>
-      <c r="I17" s="47">
-        <f>H17/H$30</f>
-        <v/>
-      </c>
-      <c r="J17" s="48" t="inlineStr">
-        <is>
-          <t>Estimado de mercado</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="34" t="inlineStr">
-        <is>
-          <t>Producción técnica</t>
-        </is>
-      </c>
-      <c r="B18" s="15" t="inlineStr">
-        <is>
-          <t>Tarima y backdrop</t>
-        </is>
-      </c>
-      <c r="C18" s="35" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="36" t="inlineStr">
-        <is>
-          <t>montaje</t>
-        </is>
-      </c>
-      <c r="E18" s="37" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="F18" s="37" t="n">
-        <v>2500000</v>
-      </c>
-      <c r="G18" s="38">
-        <f>C18*E18</f>
-        <v/>
-      </c>
-      <c r="H18" s="38">
-        <f>C18*F18</f>
-        <v/>
-      </c>
-      <c r="I18" s="39">
-        <f>H18/H$30</f>
-        <v/>
-      </c>
-      <c r="J18" s="50" t="inlineStr">
-        <is>
-          <t>Estimado de mercado</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="28" customHeight="1">
-      <c r="A19" s="41" t="inlineStr">
-        <is>
-          <t>Ambientación</t>
-        </is>
-      </c>
-      <c r="B19" s="42" t="inlineStr">
-        <is>
-          <t>Diseño floral y ambientación</t>
-        </is>
-      </c>
-      <c r="C19" s="43" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="44" t="inlineStr">
-        <is>
-          <t>servicio</t>
-        </is>
-      </c>
-      <c r="E19" s="45" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="F19" s="45" t="n">
-        <v>7000000</v>
-      </c>
-      <c r="G19" s="46">
-        <f>C19*E19</f>
-        <v/>
-      </c>
-      <c r="H19" s="46">
-        <f>C19*F19</f>
-        <v/>
-      </c>
-      <c r="I19" s="47">
-        <f>H19/H$30</f>
-        <v/>
-      </c>
-      <c r="J19" s="48" t="inlineStr">
-        <is>
-          <t>Estimado — mercado Medellín $3M a $10M</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="34" t="inlineStr">
-        <is>
-          <t>Ambientación</t>
-        </is>
-      </c>
-      <c r="B20" s="15" t="inlineStr">
-        <is>
-          <t>Mobiliario lounge, barras y mantelería</t>
-        </is>
-      </c>
-      <c r="C20" s="35" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="36" t="inlineStr">
-        <is>
-          <t>servicio</t>
-        </is>
-      </c>
-      <c r="E20" s="37" t="n">
-        <v>1500000</v>
-      </c>
-      <c r="F20" s="37" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="G20" s="38">
-        <f>C20*E20</f>
-        <v/>
-      </c>
-      <c r="H20" s="38">
-        <f>C20*F20</f>
-        <v/>
-      </c>
-      <c r="I20" s="39">
-        <f>H20/H$30</f>
-        <v/>
-      </c>
-      <c r="J20" s="50" t="inlineStr">
-        <is>
-          <t>Estimado — bajo porque Fábula ya incluye sillas y mesas</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="28" customHeight="1">
-      <c r="A21" s="41" t="inlineStr">
-        <is>
-          <t>Contenido</t>
-        </is>
-      </c>
-      <c r="B21" s="42" t="inlineStr">
-        <is>
-          <t>Fotografía · dos fotógrafas</t>
-        </is>
-      </c>
-      <c r="C21" s="43" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" s="44" t="inlineStr">
-        <is>
-          <t>servicio</t>
-        </is>
-      </c>
-      <c r="E21" s="45" t="n">
-        <v>2000000</v>
-      </c>
-      <c r="F21" s="45" t="n">
-        <v>4000000</v>
-      </c>
-      <c r="G21" s="46">
-        <f>C21*E21</f>
-        <v/>
-      </c>
-      <c r="H21" s="46">
-        <f>C21*F21</f>
-        <v/>
-      </c>
-      <c r="I21" s="47">
-        <f>H21/H$30</f>
-        <v/>
-      </c>
-      <c r="J21" s="48" t="inlineStr">
-        <is>
-          <t>Estimado — mercado Medellín $2M a $5M</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="34" t="inlineStr">
-        <is>
-          <t>Contenido</t>
-        </is>
-      </c>
-      <c r="B22" s="15" t="inlineStr">
-        <is>
-          <t>Video · equipo de dos y edición</t>
-        </is>
-      </c>
-      <c r="C22" s="35" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" s="36" t="inlineStr">
-        <is>
-          <t>servicio</t>
-        </is>
-      </c>
-      <c r="E22" s="37" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="F22" s="37" t="n">
-        <v>6000000</v>
-      </c>
-      <c r="G22" s="38">
-        <f>C22*E22</f>
-        <v/>
-      </c>
-      <c r="H22" s="38">
-        <f>C22*F22</f>
-        <v/>
-      </c>
-      <c r="I22" s="39">
-        <f>H22/H$30</f>
-        <v/>
-      </c>
-      <c r="J22" s="50" t="inlineStr">
-        <is>
-          <t>Estimado — mercado Medellín $3M a $7M</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="28" customHeight="1">
-      <c r="A23" s="41" t="inlineStr">
-        <is>
-          <t>Experiencia</t>
-        </is>
-      </c>
-      <c r="B23" s="42" t="inlineStr">
-        <is>
-          <t>Música en vivo</t>
-        </is>
-      </c>
-      <c r="C23" s="43" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="44" t="inlineStr">
-        <is>
-          <t>servicio</t>
-        </is>
-      </c>
-      <c r="E23" s="45" t="n">
-        <v>1500000</v>
-      </c>
-      <c r="F23" s="45" t="n">
-        <v>3500000</v>
-      </c>
-      <c r="G23" s="46">
-        <f>C23*E23</f>
-        <v/>
-      </c>
-      <c r="H23" s="46">
-        <f>C23*F23</f>
-        <v/>
-      </c>
-      <c r="I23" s="47">
-        <f>H23/H$30</f>
-        <v/>
-      </c>
-      <c r="J23" s="48" t="inlineStr">
-        <is>
-          <t>Estimado — mercado Medellín $3M a $8M con show completo</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="28" customHeight="1">
-      <c r="A24" s="34" t="inlineStr">
-        <is>
-          <t>Experiencia</t>
-        </is>
-      </c>
-      <c r="B24" s="15" t="inlineStr">
-        <is>
-          <t>Detalle para cada invitada</t>
-        </is>
-      </c>
-      <c r="C24" s="35">
-        <f>$B$5</f>
-        <v/>
-      </c>
-      <c r="D24" s="36" t="inlineStr">
-        <is>
-          <t>invitada</t>
-        </is>
-      </c>
-      <c r="E24" s="37" t="n">
-        <v>35000</v>
-      </c>
-      <c r="F24" s="37" t="n">
-        <v>80000</v>
-      </c>
-      <c r="G24" s="38">
-        <f>C24*E24</f>
-        <v/>
-      </c>
-      <c r="H24" s="38">
-        <f>C24*F24</f>
-        <v/>
-      </c>
-      <c r="I24" s="39">
-        <f>H24/H$30</f>
-        <v/>
-      </c>
-      <c r="J24" s="50" t="inlineStr">
-        <is>
-          <t>Estimado — define mucho el total</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="28" customHeight="1">
-      <c r="A25" s="41" t="inlineStr">
-        <is>
-          <t>Experiencia</t>
-        </is>
-      </c>
-      <c r="B25" s="42" t="inlineStr">
-        <is>
-          <t>Papelería, señalética y nombres a mano</t>
-        </is>
-      </c>
-      <c r="C25" s="43" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="44" t="inlineStr">
-        <is>
-          <t>servicio</t>
-        </is>
-      </c>
-      <c r="E25" s="45" t="n">
-        <v>600000</v>
-      </c>
-      <c r="F25" s="45" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="G25" s="46">
-        <f>C25*E25</f>
-        <v/>
-      </c>
-      <c r="H25" s="46">
-        <f>C25*F25</f>
-        <v/>
-      </c>
-      <c r="I25" s="47">
-        <f>H25/H$30</f>
-        <v/>
-      </c>
-      <c r="J25" s="48" t="inlineStr">
-        <is>
-          <t>Estimado de mercado</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="28" customHeight="1">
-      <c r="A26" s="34" t="inlineStr">
-        <is>
-          <t>Operación</t>
-        </is>
-      </c>
-      <c r="B26" s="15" t="inlineStr">
-        <is>
-          <t>Transporte y logística de montaje</t>
-        </is>
-      </c>
-      <c r="C26" s="35" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" s="36" t="inlineStr">
-        <is>
-          <t>servicio</t>
-        </is>
-      </c>
-      <c r="E26" s="37" t="n">
-        <v>800000</v>
-      </c>
-      <c r="F26" s="37" t="n">
-        <v>1500000</v>
-      </c>
-      <c r="G26" s="38">
-        <f>C26*E26</f>
-        <v/>
-      </c>
-      <c r="H26" s="38">
-        <f>C26*F26</f>
-        <v/>
-      </c>
-      <c r="I26" s="39">
-        <f>H26/H$30</f>
-        <v/>
-      </c>
-      <c r="J26" s="50" t="inlineStr">
-        <is>
-          <t>Estimado de mercado</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="51" t="inlineStr">
-        <is>
-          <t>SUBTOTAL DIRECTO</t>
-        </is>
-      </c>
-      <c r="B27" s="51" t="n"/>
-      <c r="C27" s="51" t="n"/>
-      <c r="D27" s="51" t="n"/>
-      <c r="E27" s="51" t="n"/>
-      <c r="F27" s="51" t="n"/>
-      <c r="G27" s="52">
-        <f>SUM(G8:G26)</f>
-        <v/>
-      </c>
-      <c r="H27" s="52">
-        <f>SUM(H8:H26)</f>
-        <v/>
-      </c>
-      <c r="I27" s="51" t="n"/>
-      <c r="J27" s="51" t="n"/>
-    </row>
-    <row r="28" ht="24" customHeight="1">
-      <c r="A28" s="53" t="inlineStr">
-        <is>
-          <t>Producción y dirección · Aura Productions</t>
-        </is>
-      </c>
-      <c r="B28" s="53" t="n"/>
-      <c r="C28" s="53" t="n"/>
-      <c r="D28" s="53" t="n"/>
-      <c r="E28" s="53" t="n"/>
-      <c r="F28" s="53" t="n"/>
-      <c r="G28" s="54">
-        <f>G27*$D$5</f>
-        <v/>
-      </c>
-      <c r="H28" s="54">
-        <f>H27*$D$5</f>
-        <v/>
-      </c>
-      <c r="I28" s="53" t="n"/>
-      <c r="J28" s="53" t="n"/>
-    </row>
-    <row r="29" ht="24" customHeight="1">
-      <c r="A29" s="53" t="inlineStr">
-        <is>
-          <t>Imprevistos</t>
-        </is>
-      </c>
-      <c r="B29" s="53" t="n"/>
-      <c r="C29" s="53" t="n"/>
-      <c r="D29" s="53" t="n"/>
-      <c r="E29" s="53" t="n"/>
-      <c r="F29" s="53" t="n"/>
-      <c r="G29" s="54">
-        <f>G27*$F$5</f>
-        <v/>
-      </c>
-      <c r="H29" s="54">
-        <f>H27*$F$5</f>
-        <v/>
-      </c>
-      <c r="I29" s="53" t="n"/>
-      <c r="J29" s="53" t="n"/>
-    </row>
-    <row r="30" ht="24" customHeight="1">
-      <c r="A30" s="55" t="inlineStr">
-        <is>
-          <t>TOTAL DE LA VELADA</t>
-        </is>
-      </c>
-      <c r="B30" s="55" t="n"/>
-      <c r="C30" s="55" t="n"/>
-      <c r="D30" s="55" t="n"/>
-      <c r="E30" s="55" t="n"/>
-      <c r="F30" s="55" t="n"/>
-      <c r="G30" s="56">
-        <f>G27+G28+G29</f>
-        <v/>
-      </c>
-      <c r="H30" s="56">
-        <f>H27+H28+H29</f>
-        <v/>
-      </c>
-      <c r="I30" s="55" t="n"/>
-      <c r="J30" s="55" t="n"/>
-    </row>
-    <row r="31" ht="24" customHeight="1">
-      <c r="A31" s="55" t="inlineStr">
-        <is>
-          <t>Por invitada</t>
-        </is>
-      </c>
-      <c r="B31" s="55" t="n"/>
-      <c r="C31" s="55" t="n"/>
-      <c r="D31" s="55" t="n"/>
-      <c r="E31" s="55" t="n"/>
-      <c r="F31" s="55" t="n"/>
-      <c r="G31" s="56">
-        <f>G30/$B$5</f>
-        <v/>
-      </c>
-      <c r="H31" s="56">
-        <f>H30/$B$5</f>
-        <v/>
-      </c>
-      <c r="I31" s="55" t="n"/>
-      <c r="J31" s="55" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="57" t="inlineStr">
-        <is>
-          <t>RESUMEN POR RUBRO</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="58" t="inlineStr">
-        <is>
-          <t>Rubro</t>
-        </is>
-      </c>
-      <c r="B34" s="58" t="inlineStr">
-        <is>
-          <t>Desde</t>
-        </is>
-      </c>
-      <c r="C34" s="58" t="inlineStr">
-        <is>
-          <t>Hasta</t>
-        </is>
-      </c>
-      <c r="D34" s="58" t="inlineStr">
-        <is>
-          <t>% del total</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="59" t="inlineStr">
-        <is>
-          <t>Locación</t>
-        </is>
-      </c>
-      <c r="B35" s="60">
-        <f>SUMIF($A$8:$A$26,$A35,$G$8:$G$26)</f>
-        <v/>
-      </c>
-      <c r="C35" s="60">
-        <f>SUMIF($A$8:$A$26,$A35,$H$8:$H$26)</f>
-        <v/>
-      </c>
-      <c r="D35" s="61">
-        <f>C35/$H$27</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="59" t="inlineStr">
-        <is>
-          <t>Gastronomía</t>
-        </is>
-      </c>
-      <c r="B36" s="60">
-        <f>SUMIF($A$8:$A$26,$A36,$G$8:$G$26)</f>
-        <v/>
-      </c>
-      <c r="C36" s="60">
-        <f>SUMIF($A$8:$A$26,$A36,$H$8:$H$26)</f>
-        <v/>
-      </c>
-      <c r="D36" s="61">
-        <f>C36/$H$27</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="59" t="inlineStr">
-        <is>
-          <t>Producción técnica</t>
-        </is>
-      </c>
-      <c r="B37" s="60">
-        <f>SUMIF($A$8:$A$26,$A37,$G$8:$G$26)</f>
-        <v/>
-      </c>
-      <c r="C37" s="60">
-        <f>SUMIF($A$8:$A$26,$A37,$H$8:$H$26)</f>
-        <v/>
-      </c>
-      <c r="D37" s="61">
-        <f>C37/$H$27</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="59" t="inlineStr">
-        <is>
-          <t>Ambientación</t>
-        </is>
-      </c>
-      <c r="B38" s="60">
-        <f>SUMIF($A$8:$A$26,$A38,$G$8:$G$26)</f>
-        <v/>
-      </c>
-      <c r="C38" s="60">
-        <f>SUMIF($A$8:$A$26,$A38,$H$8:$H$26)</f>
-        <v/>
-      </c>
-      <c r="D38" s="61">
-        <f>C38/$H$27</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="59" t="inlineStr">
-        <is>
-          <t>Contenido</t>
-        </is>
-      </c>
-      <c r="B39" s="60">
-        <f>SUMIF($A$8:$A$26,$A39,$G$8:$G$26)</f>
-        <v/>
-      </c>
-      <c r="C39" s="60">
-        <f>SUMIF($A$8:$A$26,$A39,$H$8:$H$26)</f>
-        <v/>
-      </c>
-      <c r="D39" s="61">
-        <f>C39/$H$27</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="59" t="inlineStr">
-        <is>
-          <t>Experiencia</t>
-        </is>
-      </c>
-      <c r="B40" s="60">
-        <f>SUMIF($A$8:$A$26,$A40,$G$8:$G$26)</f>
-        <v/>
-      </c>
-      <c r="C40" s="60">
-        <f>SUMIF($A$8:$A$26,$A40,$H$8:$H$26)</f>
-        <v/>
-      </c>
-      <c r="D40" s="61">
-        <f>C40/$H$27</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="59" t="inlineStr">
-        <is>
-          <t>Operación</t>
-        </is>
-      </c>
-      <c r="B41" s="60">
-        <f>SUMIF($A$8:$A$26,$A41,$G$8:$G$26)</f>
-        <v/>
-      </c>
-      <c r="C41" s="60">
-        <f>SUMIF($A$8:$A$26,$A41,$H$8:$H$26)</f>
-        <v/>
-      </c>
-      <c r="D41" s="61">
-        <f>C41/$H$27</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43" ht="52" customHeight="1">
-      <c r="A43" s="62" t="inlineStr">
-        <is>
-          <t>Cómo leer este presupuesto: solo las líneas marcadas CONFIRMADO en verde son precios reales de proveedor (Fábula). Todo lo demás son estimaciones de mercado de Medellín tomadas de rangos publicados para eventos de 120 a 200 personas, y deben reemplazarse por cotizaciones firmes antes de presentar un número cerrado. Las tres palancas que más mueven el total son el catering, el detalle para cada invitada y el diseño floral: ajustando esas tres se baja o se sube el presupuesto sin tocar la experiencia.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A28:F28"/>
-    <mergeCell ref="A3:J3"/>
-    <mergeCell ref="A27:F27"/>
-    <mergeCell ref="A31:F31"/>
-    <mergeCell ref="A43:J43"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A30:F30"/>
-    <mergeCell ref="A29:F29"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3781,7 +2589,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4005,7 +2813,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>